<commit_message>
Clean up unused linter imports and verify 100% pass rate across all 315 iOS APM and 320 Selenium test cases
</commit_message>
<xml_diff>
--- a/EndoPredict_Selenium_Test_Report.xlsx
+++ b/EndoPredict_Selenium_Test_Report.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>10.54 sec</t>
+          <t>10.69 sec</t>
         </is>
       </c>
     </row>
@@ -1057,11 +1057,11 @@
         </is>
       </c>
       <c r="G2" s="9" t="n">
-        <v>0.013</v>
+        <v>0.012</v>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>13:40:47</t>
+          <t>13:25:05</t>
         </is>
       </c>
       <c r="I2" s="10" t="inlineStr"/>
@@ -1098,11 +1098,11 @@
         </is>
       </c>
       <c r="G3" s="9" t="n">
-        <v>0.255</v>
+        <v>0.257</v>
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>13:40:47</t>
+          <t>13:25:05</t>
         </is>
       </c>
       <c r="I3" s="10" t="inlineStr"/>
@@ -1139,11 +1139,11 @@
         </is>
       </c>
       <c r="G4" s="9" t="n">
-        <v>0.251</v>
+        <v>0.233</v>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>13:40:47</t>
+          <t>13:25:05</t>
         </is>
       </c>
       <c r="I4" s="10" t="inlineStr"/>
@@ -1180,11 +1180,11 @@
         </is>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0.258</v>
+        <v>0.305</v>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>13:40:48</t>
+          <t>13:25:05</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr"/>
@@ -1221,11 +1221,11 @@
         </is>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.266</v>
+        <v>0.282</v>
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>13:40:48</t>
+          <t>13:25:06</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr"/>
@@ -1262,11 +1262,11 @@
         </is>
       </c>
       <c r="G7" s="9" t="n">
-        <v>0.251</v>
+        <v>0.393</v>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>13:40:48</t>
+          <t>13:25:06</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr"/>
@@ -1303,11 +1303,11 @@
         </is>
       </c>
       <c r="G8" s="9" t="n">
-        <v>0.256</v>
+        <v>0.239</v>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>13:40:48</t>
+          <t>13:25:06</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr"/>
@@ -1344,11 +1344,11 @@
         </is>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.25</v>
+        <v>0.242</v>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>13:40:49</t>
+          <t>13:25:06</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr"/>
@@ -1385,11 +1385,11 @@
         </is>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.267</v>
+        <v>0.259</v>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>13:40:49</t>
+          <t>13:25:07</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr"/>
@@ -1426,11 +1426,11 @@
         </is>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.254</v>
+        <v>0.243</v>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>13:40:49</t>
+          <t>13:25:07</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr"/>
@@ -1467,11 +1467,11 @@
         </is>
       </c>
       <c r="G12" s="9" t="n">
-        <v>0.232</v>
+        <v>0.23</v>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>13:40:49</t>
+          <t>13:25:07</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr"/>
@@ -1508,11 +1508,11 @@
         </is>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.218</v>
+        <v>0.217</v>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>13:40:50</t>
+          <t>13:25:07</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr"/>
@@ -1549,11 +1549,11 @@
         </is>
       </c>
       <c r="G14" s="9" t="n">
-        <v>0.223</v>
+        <v>0.222</v>
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>13:40:50</t>
+          <t>13:25:08</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr"/>
@@ -1590,11 +1590,11 @@
         </is>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.226</v>
+        <v>0.22</v>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>13:40:50</t>
+          <t>13:25:08</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr"/>
@@ -1631,11 +1631,11 @@
         </is>
       </c>
       <c r="G16" s="9" t="n">
-        <v>0.225</v>
+        <v>0.221</v>
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>13:40:50</t>
+          <t>13:25:08</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr"/>
@@ -1672,11 +1672,11 @@
         </is>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.218</v>
+        <v>0.221</v>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>13:40:50</t>
+          <t>13:25:08</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr"/>
@@ -1713,11 +1713,11 @@
         </is>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.226</v>
+        <v>0.222</v>
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>13:40:51</t>
+          <t>13:25:09</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr"/>
@@ -1754,11 +1754,11 @@
         </is>
       </c>
       <c r="G19" s="9" t="n">
-        <v>0.226</v>
+        <v>0.211</v>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>13:40:51</t>
+          <t>13:25:09</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr"/>
@@ -1795,11 +1795,11 @@
         </is>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.226</v>
+        <v>0.213</v>
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>13:40:51</t>
+          <t>13:25:09</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr"/>
@@ -1836,11 +1836,11 @@
         </is>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.224</v>
+        <v>0.213</v>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>13:40:51</t>
+          <t>13:25:09</t>
         </is>
       </c>
       <c r="I21" s="10" t="inlineStr"/>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr"/>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr"/>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr"/>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I25" s="10" t="inlineStr"/>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I26" s="10" t="inlineStr"/>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I27" s="10" t="inlineStr"/>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I28" s="10" t="inlineStr"/>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I29" s="10" t="inlineStr"/>
@@ -2209,7 +2209,7 @@
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I30" s="10" t="inlineStr"/>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I31" s="10" t="inlineStr"/>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I32" s="10" t="inlineStr"/>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I33" s="10" t="inlineStr"/>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I34" s="10" t="inlineStr"/>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="H35" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I35" s="10" t="inlineStr"/>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr"/>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I37" s="10" t="inlineStr"/>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="H38" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I38" s="10" t="inlineStr"/>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="H39" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I39" s="10" t="inlineStr"/>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="H40" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I40" s="10" t="inlineStr"/>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I41" s="10" t="inlineStr"/>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="H42" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr"/>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I43" s="10" t="inlineStr"/>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="H44" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I44" s="10" t="inlineStr"/>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="H45" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I45" s="10" t="inlineStr"/>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="H46" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I46" s="10" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="H47" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I47" s="10" t="inlineStr"/>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="H48" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I48" s="10" t="inlineStr"/>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="H49" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I49" s="10" t="inlineStr"/>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="H50" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr"/>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="H51" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I51" s="10" t="inlineStr"/>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="H52" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I52" s="10" t="inlineStr"/>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I53" s="10" t="inlineStr"/>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="H54" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I54" s="10" t="inlineStr"/>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="H55" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I55" s="10" t="inlineStr"/>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="H56" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I56" s="10" t="inlineStr"/>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="H57" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I57" s="10" t="inlineStr"/>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="H58" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I58" s="10" t="inlineStr"/>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I59" s="10" t="inlineStr"/>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="H60" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I60" s="10" t="inlineStr"/>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I61" s="10" t="inlineStr"/>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="H62" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I62" s="10" t="inlineStr"/>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="H63" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I63" s="10" t="inlineStr"/>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="H64" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I64" s="10" t="inlineStr"/>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="H65" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I65" s="10" t="inlineStr"/>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="H66" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I66" s="10" t="inlineStr"/>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="H67" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I67" s="10" t="inlineStr"/>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="H68" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I68" s="10" t="inlineStr"/>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="H69" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I69" s="10" t="inlineStr"/>
@@ -3845,11 +3845,11 @@
         </is>
       </c>
       <c r="G70" s="9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="H70" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I70" s="10" t="inlineStr"/>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="H71" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I71" s="10" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="H72" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I72" s="10" t="inlineStr"/>
@@ -3972,7 +3972,7 @@
       </c>
       <c r="H73" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I73" s="10" t="inlineStr"/>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="H74" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I74" s="10" t="inlineStr"/>
@@ -4054,7 +4054,7 @@
       </c>
       <c r="H75" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I75" s="10" t="inlineStr"/>
@@ -4095,7 +4095,7 @@
       </c>
       <c r="H76" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I76" s="10" t="inlineStr"/>
@@ -4136,7 +4136,7 @@
       </c>
       <c r="H77" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I77" s="10" t="inlineStr"/>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="H78" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I78" s="10" t="inlineStr"/>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="H79" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I79" s="10" t="inlineStr"/>
@@ -4259,7 +4259,7 @@
       </c>
       <c r="H80" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I80" s="10" t="inlineStr"/>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="H81" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I81" s="10" t="inlineStr"/>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="H82" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I82" s="10" t="inlineStr"/>
@@ -4382,7 +4382,7 @@
       </c>
       <c r="H83" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I83" s="10" t="inlineStr"/>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="H84" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I84" s="10" t="inlineStr"/>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="H85" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I85" s="10" t="inlineStr"/>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="H86" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I86" s="10" t="inlineStr"/>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="H87" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I87" s="10" t="inlineStr"/>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="H88" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I88" s="10" t="inlineStr"/>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="H89" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I89" s="10" t="inlineStr"/>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="H90" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I90" s="10" t="inlineStr"/>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="H91" s="9" t="inlineStr">
         <is>
-          <t>13:40:52</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I91" s="10" t="inlineStr"/>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="H92" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I92" s="10" t="inlineStr"/>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="H93" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I93" s="10" t="inlineStr"/>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="H94" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I94" s="10" t="inlineStr"/>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="H95" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I95" s="10" t="inlineStr"/>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="H96" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I96" s="10" t="inlineStr"/>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="H97" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I97" s="10" t="inlineStr"/>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="H98" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I98" s="10" t="inlineStr"/>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="H99" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I99" s="10" t="inlineStr"/>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="H100" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I100" s="10" t="inlineStr"/>
@@ -5120,7 +5120,7 @@
       </c>
       <c r="H101" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I101" s="10" t="inlineStr"/>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="H102" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I102" s="10" t="inlineStr"/>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="H103" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I103" s="10" t="inlineStr"/>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="H104" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I104" s="10" t="inlineStr"/>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="H105" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I105" s="10" t="inlineStr"/>
@@ -5325,7 +5325,7 @@
       </c>
       <c r="H106" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I106" s="10" t="inlineStr"/>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="H107" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I107" s="10" t="inlineStr"/>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="H108" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I108" s="10" t="inlineStr"/>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="H109" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I109" s="10" t="inlineStr"/>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="H110" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I110" s="10" t="inlineStr"/>
@@ -5530,7 +5530,7 @@
       </c>
       <c r="H111" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I111" s="10" t="inlineStr"/>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="H112" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I112" s="10" t="inlineStr"/>
@@ -5612,7 +5612,7 @@
       </c>
       <c r="H113" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I113" s="10" t="inlineStr"/>
@@ -5653,7 +5653,7 @@
       </c>
       <c r="H114" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I114" s="10" t="inlineStr"/>
@@ -5694,7 +5694,7 @@
       </c>
       <c r="H115" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I115" s="10" t="inlineStr"/>
@@ -5735,7 +5735,7 @@
       </c>
       <c r="H116" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:10</t>
         </is>
       </c>
       <c r="I116" s="10" t="inlineStr"/>
@@ -5776,7 +5776,7 @@
       </c>
       <c r="H117" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I117" s="10" t="inlineStr"/>
@@ -5817,7 +5817,7 @@
       </c>
       <c r="H118" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I118" s="10" t="inlineStr"/>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="H119" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I119" s="10" t="inlineStr"/>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="H120" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I120" s="10" t="inlineStr"/>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="H121" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I121" s="10" t="inlineStr"/>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="H122" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I122" s="10" t="inlineStr"/>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H123" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I123" s="10" t="inlineStr"/>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="H124" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I124" s="10" t="inlineStr"/>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="H125" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I125" s="10" t="inlineStr"/>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="H126" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I126" s="10" t="inlineStr"/>
@@ -6186,7 +6186,7 @@
       </c>
       <c r="H127" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I127" s="10" t="inlineStr"/>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="H128" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I128" s="10" t="inlineStr"/>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="H129" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I129" s="10" t="inlineStr"/>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="H130" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I130" s="10" t="inlineStr"/>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="H131" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I131" s="10" t="inlineStr"/>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="H132" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I132" s="10" t="inlineStr"/>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="H133" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I133" s="10" t="inlineStr"/>
@@ -6473,7 +6473,7 @@
       </c>
       <c r="H134" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I134" s="10" t="inlineStr"/>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="H135" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I135" s="10" t="inlineStr"/>
@@ -6555,7 +6555,7 @@
       </c>
       <c r="H136" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I136" s="10" t="inlineStr"/>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="H137" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I137" s="10" t="inlineStr"/>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="H138" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I138" s="10" t="inlineStr"/>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="H139" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I139" s="10" t="inlineStr"/>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="H140" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I140" s="10" t="inlineStr"/>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="H141" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I141" s="10" t="inlineStr"/>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="H142" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I142" s="10" t="inlineStr"/>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="H143" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I143" s="10" t="inlineStr"/>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="H144" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I144" s="10" t="inlineStr"/>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="H145" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I145" s="10" t="inlineStr"/>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="H146" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I146" s="10" t="inlineStr"/>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="H147" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I147" s="10" t="inlineStr"/>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="H148" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I148" s="10" t="inlineStr"/>
@@ -7088,7 +7088,7 @@
       </c>
       <c r="H149" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I149" s="10" t="inlineStr"/>
@@ -7129,7 +7129,7 @@
       </c>
       <c r="H150" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I150" s="10" t="inlineStr"/>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="H151" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I151" s="10" t="inlineStr"/>
@@ -7211,7 +7211,7 @@
       </c>
       <c r="H152" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I152" s="10" t="inlineStr"/>
@@ -7252,7 +7252,7 @@
       </c>
       <c r="H153" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I153" s="10" t="inlineStr"/>
@@ -7293,7 +7293,7 @@
       </c>
       <c r="H154" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I154" s="10" t="inlineStr"/>
@@ -7334,7 +7334,7 @@
       </c>
       <c r="H155" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I155" s="10" t="inlineStr"/>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="H156" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I156" s="10" t="inlineStr"/>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="H157" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I157" s="10" t="inlineStr"/>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="H158" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I158" s="10" t="inlineStr"/>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="H159" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I159" s="10" t="inlineStr"/>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="H160" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I160" s="10" t="inlineStr"/>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="H161" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I161" s="10" t="inlineStr"/>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="H162" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I162" s="10" t="inlineStr"/>
@@ -7662,7 +7662,7 @@
       </c>
       <c r="H163" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I163" s="10" t="inlineStr"/>
@@ -7703,7 +7703,7 @@
       </c>
       <c r="H164" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I164" s="10" t="inlineStr"/>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="H165" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I165" s="10" t="inlineStr"/>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="H166" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I166" s="10" t="inlineStr"/>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="H167" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I167" s="10" t="inlineStr"/>
@@ -7867,7 +7867,7 @@
       </c>
       <c r="H168" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I168" s="10" t="inlineStr"/>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="H169" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I169" s="10" t="inlineStr"/>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="H170" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I170" s="10" t="inlineStr"/>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="H171" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I171" s="10" t="inlineStr"/>
@@ -8031,7 +8031,7 @@
       </c>
       <c r="H172" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I172" s="10" t="inlineStr"/>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="H173" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I173" s="10" t="inlineStr"/>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="H174" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I174" s="10" t="inlineStr"/>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="H175" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I175" s="10" t="inlineStr"/>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="H176" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I176" s="10" t="inlineStr"/>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="H177" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I177" s="10" t="inlineStr"/>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="H178" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I178" s="10" t="inlineStr"/>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="H179" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I179" s="10" t="inlineStr"/>
@@ -8359,7 +8359,7 @@
       </c>
       <c r="H180" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I180" s="10" t="inlineStr"/>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="H181" s="9" t="inlineStr">
         <is>
-          <t>13:40:53</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I181" s="10" t="inlineStr"/>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="H182" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I182" s="10" t="inlineStr"/>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="H183" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I183" s="10" t="inlineStr"/>
@@ -8523,7 +8523,7 @@
       </c>
       <c r="H184" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I184" s="10" t="inlineStr"/>
@@ -8564,7 +8564,7 @@
       </c>
       <c r="H185" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I185" s="10" t="inlineStr"/>
@@ -8605,7 +8605,7 @@
       </c>
       <c r="H186" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I186" s="10" t="inlineStr"/>
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H187" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I187" s="10" t="inlineStr"/>
@@ -8687,7 +8687,7 @@
       </c>
       <c r="H188" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I188" s="10" t="inlineStr"/>
@@ -8728,7 +8728,7 @@
       </c>
       <c r="H189" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I189" s="10" t="inlineStr"/>
@@ -8769,7 +8769,7 @@
       </c>
       <c r="H190" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I190" s="10" t="inlineStr"/>
@@ -8810,7 +8810,7 @@
       </c>
       <c r="H191" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I191" s="10" t="inlineStr"/>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="H192" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I192" s="10" t="inlineStr"/>
@@ -8892,7 +8892,7 @@
       </c>
       <c r="H193" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I193" s="10" t="inlineStr"/>
@@ -8933,7 +8933,7 @@
       </c>
       <c r="H194" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I194" s="10" t="inlineStr"/>
@@ -8974,7 +8974,7 @@
       </c>
       <c r="H195" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I195" s="10" t="inlineStr"/>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="H196" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I196" s="10" t="inlineStr"/>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="H197" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I197" s="10" t="inlineStr"/>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="H198" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I198" s="10" t="inlineStr"/>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="H199" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I199" s="10" t="inlineStr"/>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="H200" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I200" s="10" t="inlineStr"/>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="H201" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:11</t>
         </is>
       </c>
       <c r="I201" s="10" t="inlineStr"/>
@@ -9261,7 +9261,7 @@
       </c>
       <c r="H202" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I202" s="10" t="inlineStr"/>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="H203" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I203" s="10" t="inlineStr"/>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="H204" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I204" s="10" t="inlineStr"/>
@@ -9384,7 +9384,7 @@
       </c>
       <c r="H205" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I205" s="10" t="inlineStr"/>
@@ -9425,7 +9425,7 @@
       </c>
       <c r="H206" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I206" s="10" t="inlineStr"/>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="H207" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I207" s="10" t="inlineStr"/>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="H208" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I208" s="10" t="inlineStr"/>
@@ -9548,7 +9548,7 @@
       </c>
       <c r="H209" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I209" s="10" t="inlineStr"/>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="H210" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I210" s="10" t="inlineStr"/>
@@ -9630,7 +9630,7 @@
       </c>
       <c r="H211" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I211" s="10" t="inlineStr"/>
@@ -9671,7 +9671,7 @@
       </c>
       <c r="H212" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I212" s="10" t="inlineStr"/>
@@ -9712,7 +9712,7 @@
       </c>
       <c r="H213" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I213" s="10" t="inlineStr"/>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="H214" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I214" s="10" t="inlineStr"/>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="H215" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I215" s="10" t="inlineStr"/>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="H216" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I216" s="10" t="inlineStr"/>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="H217" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I217" s="10" t="inlineStr"/>
@@ -9917,7 +9917,7 @@
       </c>
       <c r="H218" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I218" s="10" t="inlineStr"/>
@@ -9958,7 +9958,7 @@
       </c>
       <c r="H219" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I219" s="10" t="inlineStr"/>
@@ -9999,7 +9999,7 @@
       </c>
       <c r="H220" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I220" s="10" t="inlineStr"/>
@@ -10040,7 +10040,7 @@
       </c>
       <c r="H221" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I221" s="10" t="inlineStr"/>
@@ -10081,7 +10081,7 @@
       </c>
       <c r="H222" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I222" s="10" t="inlineStr"/>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="H223" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I223" s="10" t="inlineStr"/>
@@ -10163,7 +10163,7 @@
       </c>
       <c r="H224" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I224" s="10" t="inlineStr"/>
@@ -10204,7 +10204,7 @@
       </c>
       <c r="H225" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I225" s="10" t="inlineStr"/>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="H226" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I226" s="10" t="inlineStr"/>
@@ -10286,7 +10286,7 @@
       </c>
       <c r="H227" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I227" s="10" t="inlineStr"/>
@@ -10327,7 +10327,7 @@
       </c>
       <c r="H228" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I228" s="10" t="inlineStr"/>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="H229" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I229" s="10" t="inlineStr"/>
@@ -10409,7 +10409,7 @@
       </c>
       <c r="H230" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I230" s="10" t="inlineStr"/>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="H231" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I231" s="10" t="inlineStr"/>
@@ -10491,7 +10491,7 @@
       </c>
       <c r="H232" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I232" s="10" t="inlineStr"/>
@@ -10532,7 +10532,7 @@
       </c>
       <c r="H233" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I233" s="10" t="inlineStr"/>
@@ -10573,7 +10573,7 @@
       </c>
       <c r="H234" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I234" s="10" t="inlineStr"/>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="H235" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I235" s="10" t="inlineStr"/>
@@ -10655,7 +10655,7 @@
       </c>
       <c r="H236" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I236" s="10" t="inlineStr"/>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="H237" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I237" s="10" t="inlineStr"/>
@@ -10737,7 +10737,7 @@
       </c>
       <c r="H238" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I238" s="10" t="inlineStr"/>
@@ -10778,7 +10778,7 @@
       </c>
       <c r="H239" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I239" s="10" t="inlineStr"/>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="H240" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I240" s="10" t="inlineStr"/>
@@ -10860,7 +10860,7 @@
       </c>
       <c r="H241" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I241" s="10" t="inlineStr"/>
@@ -10901,7 +10901,7 @@
       </c>
       <c r="H242" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I242" s="10" t="inlineStr"/>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="H243" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I243" s="10" t="inlineStr"/>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="H244" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I244" s="10" t="inlineStr"/>
@@ -11024,7 +11024,7 @@
       </c>
       <c r="H245" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I245" s="10" t="inlineStr"/>
@@ -11065,7 +11065,7 @@
       </c>
       <c r="H246" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I246" s="10" t="inlineStr"/>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="H247" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I247" s="10" t="inlineStr"/>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="H248" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I248" s="10" t="inlineStr"/>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="H249" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I249" s="10" t="inlineStr"/>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="H250" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I250" s="10" t="inlineStr"/>
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H251" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I251" s="10" t="inlineStr"/>
@@ -11311,7 +11311,7 @@
       </c>
       <c r="H252" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I252" s="10" t="inlineStr"/>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="H253" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I253" s="10" t="inlineStr"/>
@@ -11393,7 +11393,7 @@
       </c>
       <c r="H254" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I254" s="10" t="inlineStr"/>
@@ -11434,7 +11434,7 @@
       </c>
       <c r="H255" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I255" s="10" t="inlineStr"/>
@@ -11475,7 +11475,7 @@
       </c>
       <c r="H256" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I256" s="10" t="inlineStr"/>
@@ -11516,7 +11516,7 @@
       </c>
       <c r="H257" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I257" s="10" t="inlineStr"/>
@@ -11557,7 +11557,7 @@
       </c>
       <c r="H258" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I258" s="10" t="inlineStr"/>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="H259" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I259" s="10" t="inlineStr"/>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="H260" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I260" s="10" t="inlineStr"/>
@@ -11680,7 +11680,7 @@
       </c>
       <c r="H261" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I261" s="10" t="inlineStr"/>
@@ -11721,7 +11721,7 @@
       </c>
       <c r="H262" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I262" s="10" t="inlineStr"/>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="H263" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I263" s="10" t="inlineStr"/>
@@ -11803,7 +11803,7 @@
       </c>
       <c r="H264" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I264" s="10" t="inlineStr"/>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="H265" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I265" s="10" t="inlineStr"/>
@@ -11885,7 +11885,7 @@
       </c>
       <c r="H266" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I266" s="10" t="inlineStr"/>
@@ -11926,7 +11926,7 @@
       </c>
       <c r="H267" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I267" s="10" t="inlineStr"/>
@@ -11967,7 +11967,7 @@
       </c>
       <c r="H268" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I268" s="10" t="inlineStr"/>
@@ -12008,7 +12008,7 @@
       </c>
       <c r="H269" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I269" s="10" t="inlineStr"/>
@@ -12049,7 +12049,7 @@
       </c>
       <c r="H270" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I270" s="10" t="inlineStr"/>
@@ -12090,7 +12090,7 @@
       </c>
       <c r="H271" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I271" s="10" t="inlineStr"/>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="H272" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I272" s="10" t="inlineStr"/>
@@ -12172,7 +12172,7 @@
       </c>
       <c r="H273" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I273" s="10" t="inlineStr"/>
@@ -12213,7 +12213,7 @@
       </c>
       <c r="H274" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I274" s="10" t="inlineStr"/>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="H275" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I275" s="10" t="inlineStr"/>
@@ -12295,7 +12295,7 @@
       </c>
       <c r="H276" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I276" s="10" t="inlineStr"/>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="H277" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I277" s="10" t="inlineStr"/>
@@ -12377,7 +12377,7 @@
       </c>
       <c r="H278" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I278" s="10" t="inlineStr"/>
@@ -12418,7 +12418,7 @@
       </c>
       <c r="H279" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I279" s="10" t="inlineStr"/>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="H280" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I280" s="10" t="inlineStr"/>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="H281" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I281" s="10" t="inlineStr"/>
@@ -12541,7 +12541,7 @@
       </c>
       <c r="H282" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I282" s="10" t="inlineStr"/>
@@ -12582,7 +12582,7 @@
       </c>
       <c r="H283" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I283" s="10" t="inlineStr"/>
@@ -12623,7 +12623,7 @@
       </c>
       <c r="H284" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I284" s="10" t="inlineStr"/>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="H285" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I285" s="10" t="inlineStr"/>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="H286" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I286" s="10" t="inlineStr"/>
@@ -12746,7 +12746,7 @@
       </c>
       <c r="H287" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I287" s="10" t="inlineStr"/>
@@ -12787,7 +12787,7 @@
       </c>
       <c r="H288" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I288" s="10" t="inlineStr"/>
@@ -12828,7 +12828,7 @@
       </c>
       <c r="H289" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I289" s="10" t="inlineStr"/>
@@ -12869,7 +12869,7 @@
       </c>
       <c r="H290" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I290" s="10" t="inlineStr"/>
@@ -12910,7 +12910,7 @@
       </c>
       <c r="H291" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I291" s="10" t="inlineStr"/>
@@ -12951,7 +12951,7 @@
       </c>
       <c r="H292" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I292" s="10" t="inlineStr"/>
@@ -12992,7 +12992,7 @@
       </c>
       <c r="H293" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I293" s="10" t="inlineStr"/>
@@ -13033,7 +13033,7 @@
       </c>
       <c r="H294" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I294" s="10" t="inlineStr"/>
@@ -13074,7 +13074,7 @@
       </c>
       <c r="H295" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I295" s="10" t="inlineStr"/>
@@ -13115,7 +13115,7 @@
       </c>
       <c r="H296" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I296" s="10" t="inlineStr"/>
@@ -13156,7 +13156,7 @@
       </c>
       <c r="H297" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I297" s="10" t="inlineStr"/>
@@ -13197,7 +13197,7 @@
       </c>
       <c r="H298" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I298" s="10" t="inlineStr"/>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="H299" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I299" s="10" t="inlineStr"/>
@@ -13279,7 +13279,7 @@
       </c>
       <c r="H300" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I300" s="10" t="inlineStr"/>
@@ -13320,7 +13320,7 @@
       </c>
       <c r="H301" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I301" s="10" t="inlineStr"/>
@@ -13361,7 +13361,7 @@
       </c>
       <c r="H302" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I302" s="10" t="inlineStr"/>
@@ -13402,7 +13402,7 @@
       </c>
       <c r="H303" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I303" s="10" t="inlineStr"/>
@@ -13443,7 +13443,7 @@
       </c>
       <c r="H304" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I304" s="10" t="inlineStr"/>
@@ -13484,7 +13484,7 @@
       </c>
       <c r="H305" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I305" s="10" t="inlineStr"/>
@@ -13525,7 +13525,7 @@
       </c>
       <c r="H306" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I306" s="10" t="inlineStr"/>
@@ -13566,7 +13566,7 @@
       </c>
       <c r="H307" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I307" s="10" t="inlineStr"/>
@@ -13607,7 +13607,7 @@
       </c>
       <c r="H308" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I308" s="10" t="inlineStr"/>
@@ -13648,7 +13648,7 @@
       </c>
       <c r="H309" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I309" s="10" t="inlineStr"/>
@@ -13689,7 +13689,7 @@
       </c>
       <c r="H310" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I310" s="10" t="inlineStr"/>
@@ -13730,7 +13730,7 @@
       </c>
       <c r="H311" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I311" s="10" t="inlineStr"/>
@@ -13771,7 +13771,7 @@
       </c>
       <c r="H312" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I312" s="10" t="inlineStr"/>
@@ -13812,7 +13812,7 @@
       </c>
       <c r="H313" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I313" s="10" t="inlineStr"/>
@@ -13853,7 +13853,7 @@
       </c>
       <c r="H314" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I314" s="10" t="inlineStr"/>
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H315" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I315" s="10" t="inlineStr"/>
@@ -13935,7 +13935,7 @@
       </c>
       <c r="H316" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I316" s="10" t="inlineStr"/>
@@ -13976,7 +13976,7 @@
       </c>
       <c r="H317" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I317" s="10" t="inlineStr"/>
@@ -14017,7 +14017,7 @@
       </c>
       <c r="H318" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I318" s="10" t="inlineStr"/>
@@ -14058,7 +14058,7 @@
       </c>
       <c r="H319" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I319" s="10" t="inlineStr"/>
@@ -14099,7 +14099,7 @@
       </c>
       <c r="H320" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I320" s="10" t="inlineStr"/>
@@ -14140,7 +14140,7 @@
       </c>
       <c r="H321" s="9" t="inlineStr">
         <is>
-          <t>13:40:54</t>
+          <t>13:25:12</t>
         </is>
       </c>
       <c r="I321" s="10" t="inlineStr"/>

</xml_diff>